<commit_message>
Complete label detection examples
</commit_message>
<xml_diff>
--- a/examples/micro_workbooks/label_detection.xlsx
+++ b/examples/micro_workbooks/label_detection.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\chris\Software\excel-grapher\examples\micro_workbooks\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6353F738-9945-43EB-B355-607884ED42CA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CE4F8D8E-BE7A-4FEE-AF9F-4BE52089A565}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="12015" yWindow="0" windowWidth="11985" windowHeight="12780" xr2:uid="{55BB74E6-7BE9-4E5B-B38A-AC356C7BC3EA}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="56" uniqueCount="34">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="61" uniqueCount="39">
   <si>
     <t>Row 1</t>
   </si>
@@ -141,13 +141,28 @@
   </si>
   <si>
     <t>Source: CIA Factbook, 2012</t>
+  </si>
+  <si>
+    <t>Country Details</t>
+  </si>
+  <si>
+    <t>United States</t>
+  </si>
+  <si>
+    <t>Nominal</t>
+  </si>
+  <si>
+    <t>Real</t>
+  </si>
+  <si>
+    <t>GDP ($)</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -157,6 +172,22 @@
     </font>
     <font>
       <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <i/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -184,9 +215,16 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" indent="2"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -507,7 +545,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DD4DDA74-4528-4F1F-AF4F-5F8ACA610B06}">
-  <dimension ref="A1:E49"/>
+  <dimension ref="A1:E56"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.25">
@@ -618,10 +656,10 @@
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A15" s="1"/>
-      <c r="C15" s="3" t="s">
+      <c r="C15" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="D15" s="3"/>
+      <c r="D15" s="6"/>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A16" s="1"/>
@@ -633,7 +671,7 @@
       </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A17" s="2" t="s">
+      <c r="A17" s="5" t="s">
         <v>24</v>
       </c>
       <c r="B17" s="1" t="s">
@@ -647,7 +685,7 @@
       </c>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A18" s="2"/>
+      <c r="A18" s="5"/>
       <c r="B18" s="1" t="s">
         <v>26</v>
       </c>
@@ -889,9 +927,49 @@
         <v>19</v>
       </c>
     </row>
-    <row r="49" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
         <v>33</v>
+      </c>
+    </row>
+    <row r="51" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A51" s="3" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="52" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A52" s="3"/>
+      <c r="B52">
+        <v>2010</v>
+      </c>
+    </row>
+    <row r="53" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A53" s="1" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="54" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A54" s="2" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="55" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A55" s="4" t="s">
+        <v>36</v>
+      </c>
+      <c r="B55">
+        <v>15.01</v>
+      </c>
+      <c r="E55">
+        <v>2010</v>
+      </c>
+    </row>
+    <row r="56" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A56" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="B56">
+        <v>15.31</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Change names of default behaviors
</commit_message>
<xml_diff>
--- a/examples/micro_workbooks/label_detection.xlsx
+++ b/examples/micro_workbooks/label_detection.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\chris\Software\excel-grapher\examples\micro_workbooks\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CE4F8D8E-BE7A-4FEE-AF9F-4BE52089A565}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{314BEF1F-6D5A-4FE2-A26A-9092DB030A09}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="12015" yWindow="0" windowWidth="11985" windowHeight="12780" xr2:uid="{55BB74E6-7BE9-4E5B-B38A-AC356C7BC3EA}"/>
   </bookViews>
@@ -927,44 +927,41 @@
         <v>19</v>
       </c>
     </row>
-    <row r="49" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="51" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A51" s="3" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="52" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A52" s="3"/>
       <c r="B52">
         <v>2010</v>
       </c>
     </row>
-    <row r="53" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A53" s="1" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="54" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A54" s="2" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="55" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A55" s="4" t="s">
         <v>36</v>
       </c>
       <c r="B55">
         <v>15.01</v>
       </c>
-      <c r="E55">
-        <v>2010</v>
-      </c>
-    </row>
-    <row r="56" spans="1:5" x14ac:dyDescent="0.25">
+    </row>
+    <row r="56" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A56" s="4" t="s">
         <v>37</v>
       </c>

</xml_diff>